<commit_message>
update: made sure all test cases are present in the new version
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/ROUND_ROUNDUP_ROUNDDOWN.xlsx
+++ b/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/ROUND_ROUNDUP_ROUNDDOWN.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5297CF-EC5F-4152-99CE-A303A6A2C9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C306F692-B903-416F-99EE-AEB7F42C2BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -188,7 +188,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -307,7 +307,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
@@ -315,15 +315,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -1783,22 +1782,22 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A56" s="7">
+      <c r="A56">
         <v>2.5</v>
       </c>
-      <c r="B56" s="7">
-        <v>0</v>
-      </c>
-      <c r="C56" s="12">
-        <f>ROUND(A56,B56)</f>
+      <c r="B56">
+        <v>0</v>
+      </c>
+      <c r="C56" s="11">
+        <f t="shared" ref="C56:C91" si="24">ROUND(A56,B56)</f>
         <v>3</v>
       </c>
-      <c r="D56" s="12">
-        <f>ROUNDUP(A56,B56)</f>
+      <c r="D56" s="11">
+        <f t="shared" ref="D56:D91" si="25">ROUNDUP(A56,B56)</f>
         <v>3</v>
       </c>
-      <c r="E56" s="14">
-        <f>ROUNDDOWN(A56,B56)</f>
+      <c r="E56" s="13">
+        <f t="shared" ref="E56:E91" si="26">ROUNDDOWN(A56,B56)</f>
         <v>2</v>
       </c>
       <c r="F56" t="s">
@@ -1806,82 +1805,82 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A57" s="7">
+      <c r="A57">
         <v>-2.5</v>
       </c>
-      <c r="B57" s="7">
-        <v>0</v>
-      </c>
-      <c r="C57" s="13">
-        <f>ROUND(A57,B57)</f>
+      <c r="B57">
+        <v>0</v>
+      </c>
+      <c r="C57" s="12">
+        <f t="shared" si="24"/>
         <v>-3</v>
       </c>
-      <c r="D57" s="13">
-        <f>ROUNDUP(A57,B57)</f>
+      <c r="D57" s="12">
+        <f t="shared" si="25"/>
         <v>-3</v>
       </c>
-      <c r="E57" s="15">
-        <f>ROUNDDOWN(A57,B57)</f>
+      <c r="E57" s="14">
+        <f t="shared" si="26"/>
         <v>-2</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A58" s="7">
+      <c r="A58">
         <v>0.5</v>
       </c>
-      <c r="B58" s="7">
-        <v>0</v>
-      </c>
-      <c r="C58" s="12">
-        <f>ROUND(A58,B58)</f>
-        <v>1</v>
-      </c>
-      <c r="D58" s="12">
-        <f>ROUNDUP(A58,B58)</f>
-        <v>1</v>
-      </c>
-      <c r="E58" s="14">
-        <f>ROUNDDOWN(A58,B58)</f>
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58" s="11">
+        <f t="shared" si="24"/>
+        <v>1</v>
+      </c>
+      <c r="D58" s="11">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
+      <c r="E58" s="13">
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A59" s="7">
+      <c r="A59">
         <v>-0.5</v>
       </c>
-      <c r="B59" s="7">
-        <v>0</v>
-      </c>
-      <c r="C59" s="12">
-        <f>ROUND(A59,B59)</f>
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59" s="11">
+        <f t="shared" si="24"/>
         <v>-1</v>
       </c>
-      <c r="D59" s="12">
-        <f>ROUNDUP(A59,B59)</f>
+      <c r="D59" s="11">
+        <f t="shared" si="25"/>
         <v>-1</v>
       </c>
-      <c r="E59" s="14">
-        <f>ROUNDDOWN(A59,B59)</f>
+      <c r="E59" s="13">
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A60" s="7">
+      <c r="A60">
         <v>2.6749999999999998</v>
       </c>
-      <c r="B60" s="7">
-        <v>2</v>
-      </c>
-      <c r="C60" s="12">
-        <f>ROUND(A60,B60)</f>
+      <c r="B60">
+        <v>2</v>
+      </c>
+      <c r="C60" s="11">
+        <f t="shared" si="24"/>
         <v>2.68</v>
       </c>
-      <c r="D60" s="12">
-        <f>ROUNDUP(A60,B60)</f>
+      <c r="D60" s="11">
+        <f t="shared" si="25"/>
         <v>2.6799999999999997</v>
       </c>
-      <c r="E60" s="14">
-        <f>ROUNDDOWN(A60,B60)</f>
+      <c r="E60" s="13">
+        <f t="shared" si="26"/>
         <v>2.67</v>
       </c>
       <c r="F60" t="s">
@@ -1889,62 +1888,62 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A61" s="7">
+      <c r="A61">
         <v>1.0049999999999999</v>
       </c>
-      <c r="B61" s="7">
-        <v>2</v>
-      </c>
-      <c r="C61" s="12">
-        <f>ROUND(A61,B61)</f>
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61" s="11">
+        <f t="shared" si="24"/>
         <v>1.01</v>
       </c>
-      <c r="D61" s="12">
-        <f>ROUNDUP(A61,B61)</f>
+      <c r="D61" s="11">
+        <f t="shared" si="25"/>
         <v>1.01</v>
       </c>
-      <c r="E61" s="14">
-        <f>ROUNDDOWN(A61,B61)</f>
+      <c r="E61" s="13">
+        <f t="shared" si="26"/>
         <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A62" s="7">
+      <c r="A62">
         <v>-1.0049999999999999</v>
       </c>
-      <c r="B62" s="7">
-        <v>2</v>
-      </c>
-      <c r="C62" s="12">
-        <f>ROUND(A62,B62)</f>
+      <c r="B62">
+        <v>2</v>
+      </c>
+      <c r="C62" s="11">
+        <f t="shared" si="24"/>
         <v>-1.01</v>
       </c>
-      <c r="D62" s="12">
-        <f>ROUNDUP(A62,B62)</f>
+      <c r="D62" s="11">
+        <f t="shared" si="25"/>
         <v>-1.01</v>
       </c>
-      <c r="E62" s="14">
-        <f>ROUNDDOWN(A62,B62)</f>
+      <c r="E62" s="13">
+        <f t="shared" si="26"/>
         <v>-1</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A63" s="7">
+      <c r="A63">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B63" s="7">
-        <v>1</v>
-      </c>
-      <c r="C63" s="12">
-        <f>ROUND(A63,B63)</f>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" s="11">
+        <f t="shared" si="24"/>
         <v>1.1000000000000001</v>
       </c>
-      <c r="D63" s="12">
-        <f>ROUNDUP(A63,B63)</f>
+      <c r="D63" s="11">
+        <f t="shared" si="25"/>
         <v>1.1000000000000001</v>
       </c>
-      <c r="E63" s="14">
-        <f>ROUNDDOWN(A63,B63)</f>
+      <c r="E63" s="13">
+        <f t="shared" si="26"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="F63" t="s">
@@ -1952,23 +1951,23 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A64" s="7">
+      <c r="A64">
         <f>0.1+0.2</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="B64" s="7">
-        <v>1</v>
-      </c>
-      <c r="C64" s="12">
-        <f>ROUND(A64,B64)</f>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" s="11">
+        <f t="shared" si="24"/>
         <v>0.3</v>
       </c>
-      <c r="D64" s="12">
-        <f>ROUNDUP(A64,B64)</f>
+      <c r="D64" s="11">
+        <f t="shared" si="25"/>
         <v>0.3</v>
       </c>
-      <c r="E64" s="14">
-        <f>ROUNDDOWN(A64,B64)</f>
+      <c r="E64" s="13">
+        <f t="shared" si="26"/>
         <v>0.3</v>
       </c>
       <c r="F64" s="6" t="s">
@@ -1976,23 +1975,23 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A65" s="7">
+      <c r="A65">
         <f>1-0.9</f>
         <v>9.9999999999999978E-2</v>
       </c>
-      <c r="B65" s="7">
-        <v>1</v>
-      </c>
-      <c r="C65" s="12">
-        <f>ROUND(A65,B65)</f>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" s="11">
+        <f t="shared" si="24"/>
         <v>0.1</v>
       </c>
-      <c r="D65" s="12">
-        <f>ROUNDUP(A65,B65)</f>
+      <c r="D65" s="11">
+        <f t="shared" si="25"/>
         <v>0.1</v>
       </c>
-      <c r="E65" s="14">
-        <f>ROUNDDOWN(A65,B65)</f>
+      <c r="E65" s="13">
+        <f t="shared" si="26"/>
         <v>0.1</v>
       </c>
       <c r="F65" s="6" t="s">
@@ -2000,462 +1999,448 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A66" s="7">
+      <c r="A66">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="B66" s="7">
+      <c r="B66">
         <v>15</v>
       </c>
-      <c r="C66" s="12">
-        <f>ROUND(A66,B66)</f>
+      <c r="C66" s="11">
+        <f t="shared" si="24"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="D66" s="12">
-        <f>ROUNDUP(A66,B66)</f>
+      <c r="D66" s="11">
+        <f t="shared" si="25"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="E66" s="14">
-        <f>ROUNDDOWN(A66,B66)</f>
+      <c r="E66" s="13">
+        <f t="shared" si="26"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="F66" s="7" t="s">
+      <c r="F66" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A67" s="7">
+      <c r="A67">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="B67" s="7">
+      <c r="B67">
         <v>16</v>
       </c>
-      <c r="C67" s="12">
-        <f>ROUND(A67,B67)</f>
+      <c r="C67" s="11">
+        <f t="shared" si="24"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="D67" s="12">
-        <f>ROUNDUP(A67,B67)</f>
+      <c r="D67" s="11">
+        <f t="shared" si="25"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="E67" s="14">
-        <f>ROUNDDOWN(A67,B67)</f>
+      <c r="E67" s="13">
+        <f t="shared" si="26"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="F67" s="7"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A68" s="7">
+      <c r="A68">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="B68" s="7">
+      <c r="B68">
         <v>20</v>
       </c>
-      <c r="C68" s="12">
-        <f>ROUND(A68,B68)</f>
+      <c r="C68" s="11">
+        <f t="shared" si="24"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="D68" s="12">
-        <f>ROUNDUP(A68,B68)</f>
+      <c r="D68" s="11">
+        <f t="shared" si="25"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="E68" s="14">
-        <f>ROUNDDOWN(A68,B68)</f>
+      <c r="E68" s="13">
+        <f t="shared" si="26"/>
         <v>0.33333333333333298</v>
       </c>
-      <c r="F68" s="7"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A69" s="7">
+      <c r="A69">
         <v>9.9949999999999992</v>
       </c>
-      <c r="B69" s="7">
-        <v>2</v>
-      </c>
-      <c r="C69" s="12">
-        <f>ROUND(A69,B69)</f>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" s="11">
+        <f t="shared" si="24"/>
         <v>10</v>
       </c>
-      <c r="D69" s="12">
-        <f>ROUNDUP(A69,B69)</f>
+      <c r="D69" s="11">
+        <f t="shared" si="25"/>
         <v>10</v>
       </c>
-      <c r="E69" s="14">
-        <f>ROUNDDOWN(A69,B69)</f>
+      <c r="E69" s="13">
+        <f t="shared" si="26"/>
         <v>9.99</v>
       </c>
-      <c r="F69" s="7" t="s">
+      <c r="F69" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A70" s="7">
+      <c r="A70">
         <v>999.5</v>
       </c>
-      <c r="B70" s="7">
-        <v>0</v>
-      </c>
-      <c r="C70" s="12">
-        <f>ROUND(A70,B70)</f>
+      <c r="B70">
+        <v>0</v>
+      </c>
+      <c r="C70" s="11">
+        <f t="shared" si="24"/>
         <v>1000</v>
       </c>
-      <c r="D70" s="12">
-        <f>ROUNDUP(A70,B70)</f>
+      <c r="D70" s="11">
+        <f t="shared" si="25"/>
         <v>1000</v>
       </c>
-      <c r="E70" s="14">
-        <f>ROUNDDOWN(A70,B70)</f>
+      <c r="E70" s="13">
+        <f t="shared" si="26"/>
         <v>999</v>
       </c>
-      <c r="F70" s="7"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A71" s="7">
+      <c r="A71">
         <v>-9.9949999999999992</v>
       </c>
-      <c r="B71" s="7">
-        <v>2</v>
-      </c>
-      <c r="C71" s="12">
-        <f>ROUND(A71,B71)</f>
+      <c r="B71">
+        <v>2</v>
+      </c>
+      <c r="C71" s="11">
+        <f t="shared" si="24"/>
         <v>-10</v>
       </c>
-      <c r="D71" s="12">
-        <f>ROUNDUP(A71,B71)</f>
+      <c r="D71" s="11">
+        <f t="shared" si="25"/>
         <v>-10</v>
       </c>
-      <c r="E71" s="14">
-        <f>ROUNDDOWN(A71,B71)</f>
+      <c r="E71" s="13">
+        <f t="shared" si="26"/>
         <v>-9.99</v>
       </c>
-      <c r="F71" s="7"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A72" s="7">
+      <c r="A72">
         <v>9.9909999999999997</v>
       </c>
-      <c r="B72" s="7">
-        <v>2</v>
-      </c>
-      <c r="C72" s="12">
-        <f>ROUND(A72,B72)</f>
+      <c r="B72">
+        <v>2</v>
+      </c>
+      <c r="C72" s="11">
+        <f t="shared" si="24"/>
         <v>9.99</v>
       </c>
-      <c r="D72" s="12">
-        <f>ROUNDUP(A72,B72)</f>
+      <c r="D72" s="11">
+        <f t="shared" si="25"/>
         <v>10</v>
       </c>
-      <c r="E72" s="14">
-        <f>ROUNDDOWN(A72,B72)</f>
+      <c r="E72" s="13">
+        <f t="shared" si="26"/>
         <v>9.99</v>
       </c>
-      <c r="F72" s="7"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A73" s="7">
+      <c r="A73">
         <v>500</v>
       </c>
-      <c r="B73" s="7">
+      <c r="B73">
         <v>-3</v>
       </c>
-      <c r="C73" s="12">
-        <f>ROUND(A73,B73)</f>
+      <c r="C73" s="11">
+        <f t="shared" si="24"/>
         <v>1000</v>
       </c>
-      <c r="D73" s="12">
-        <f>ROUNDUP(A73,B73)</f>
+      <c r="D73" s="11">
+        <f t="shared" si="25"/>
         <v>1000</v>
       </c>
-      <c r="E73" s="14">
-        <f>ROUNDDOWN(A73,B73)</f>
-        <v>0</v>
-      </c>
-      <c r="F73" s="7" t="s">
+      <c r="E73" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="F73" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A74" s="7">
+      <c r="A74">
         <v>499</v>
       </c>
-      <c r="B74" s="7">
+      <c r="B74">
         <v>-3</v>
       </c>
-      <c r="C74" s="12">
-        <f>ROUND(A74,B74)</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="12">
-        <f>ROUNDUP(A74,B74)</f>
+      <c r="C74" s="11">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="D74" s="11">
+        <f t="shared" si="25"/>
         <v>1000</v>
       </c>
-      <c r="E74" s="14">
-        <f>ROUNDDOWN(A74,B74)</f>
-        <v>0</v>
-      </c>
-      <c r="F74" s="7"/>
+      <c r="E74" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A75" s="7">
+      <c r="A75">
         <v>-500</v>
       </c>
-      <c r="B75" s="7">
+      <c r="B75">
         <v>-3</v>
       </c>
-      <c r="C75" s="12">
-        <f>ROUND(A75,B75)</f>
+      <c r="C75" s="11">
+        <f t="shared" si="24"/>
         <v>-1000</v>
       </c>
-      <c r="D75" s="12">
-        <f>ROUNDUP(A75,B75)</f>
+      <c r="D75" s="11">
+        <f t="shared" si="25"/>
         <v>-1000</v>
       </c>
-      <c r="E75" s="14">
-        <f>ROUNDDOWN(A75,B75)</f>
-        <v>0</v>
-      </c>
-      <c r="F75" s="7"/>
+      <c r="E75" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A76" s="7">
-        <v>1</v>
-      </c>
-      <c r="B76" s="7">
+      <c r="A76">
+        <v>1</v>
+      </c>
+      <c r="B76">
         <v>-1</v>
       </c>
-      <c r="C76" s="12">
-        <f>ROUND(A76,B76)</f>
-        <v>0</v>
-      </c>
-      <c r="D76" s="12">
-        <f>ROUNDUP(A76,B76)</f>
+      <c r="C76" s="11">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="D76" s="11">
+        <f t="shared" si="25"/>
         <v>10</v>
       </c>
-      <c r="E76" s="14">
-        <f>ROUNDDOWN(A76,B76)</f>
-        <v>0</v>
-      </c>
-      <c r="F76" s="7"/>
+      <c r="E76" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A77" s="7">
+      <c r="A77">
         <v>999</v>
       </c>
-      <c r="B77" s="7">
+      <c r="B77">
         <v>-3</v>
       </c>
-      <c r="C77" s="12">
-        <f>ROUND(A77,B77)</f>
+      <c r="C77" s="11">
+        <f t="shared" si="24"/>
         <v>1000</v>
       </c>
-      <c r="D77" s="12">
-        <f>ROUNDUP(A77,B77)</f>
+      <c r="D77" s="11">
+        <f t="shared" si="25"/>
         <v>1000</v>
       </c>
-      <c r="E77" s="14">
-        <f>ROUNDDOWN(A77,B77)</f>
-        <v>0</v>
-      </c>
-      <c r="F77" s="7"/>
+      <c r="E77" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A78" s="7">
+      <c r="A78">
         <v>5</v>
       </c>
-      <c r="B78" s="7">
-        <v>0</v>
-      </c>
-      <c r="C78" s="12">
-        <f>ROUND(A78,B78)</f>
+      <c r="B78">
+        <v>0</v>
+      </c>
+      <c r="C78" s="11">
+        <f t="shared" si="24"/>
         <v>5</v>
       </c>
-      <c r="D78" s="12">
-        <f>ROUNDUP(A78,B78)</f>
+      <c r="D78" s="11">
+        <f t="shared" si="25"/>
         <v>5</v>
       </c>
-      <c r="E78" s="14">
-        <f>ROUNDDOWN(A78,B78)</f>
+      <c r="E78" s="13">
+        <f t="shared" si="26"/>
         <v>5</v>
       </c>
-      <c r="F78" s="7" t="s">
+      <c r="F78" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A79" s="7">
+      <c r="A79">
         <v>1.75</v>
       </c>
-      <c r="B79" s="7">
-        <v>2</v>
-      </c>
-      <c r="C79" s="12">
-        <f>ROUND(A79,B79)</f>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" s="11">
+        <f t="shared" si="24"/>
         <v>1.75</v>
       </c>
-      <c r="D79" s="12">
-        <f>ROUNDUP(A79,B79)</f>
+      <c r="D79" s="11">
+        <f t="shared" si="25"/>
         <v>1.75</v>
       </c>
-      <c r="E79" s="14">
-        <f>ROUNDDOWN(A79,B79)</f>
+      <c r="E79" s="13">
+        <f t="shared" si="26"/>
         <v>1.75</v>
       </c>
-      <c r="F79" s="7"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A80" s="7">
+      <c r="A80">
         <v>-1.75</v>
       </c>
-      <c r="B80" s="7">
-        <v>2</v>
-      </c>
-      <c r="C80" s="12">
-        <f>ROUND(A80,B80)</f>
+      <c r="B80">
+        <v>2</v>
+      </c>
+      <c r="C80" s="11">
+        <f t="shared" si="24"/>
         <v>-1.75</v>
       </c>
-      <c r="D80" s="12">
-        <f>ROUNDUP(A80,B80)</f>
+      <c r="D80" s="11">
+        <f t="shared" si="25"/>
         <v>-1.75</v>
       </c>
-      <c r="E80" s="14">
-        <f>ROUNDDOWN(A80,B80)</f>
+      <c r="E80" s="13">
+        <f t="shared" si="26"/>
         <v>-1.75</v>
       </c>
-      <c r="F80" s="7"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A81" s="7">
+      <c r="A81">
         <v>-1E-3</v>
       </c>
-      <c r="B81" s="7">
-        <v>2</v>
-      </c>
-      <c r="C81" s="12">
-        <f>ROUND(A81,B81)</f>
-        <v>0</v>
-      </c>
-      <c r="D81" s="12">
-        <f>ROUNDUP(A81,B81)</f>
+      <c r="B81">
+        <v>2</v>
+      </c>
+      <c r="C81" s="11">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="D81" s="11">
+        <f t="shared" si="25"/>
         <v>-0.01</v>
       </c>
-      <c r="E81" s="14">
-        <f>ROUNDDOWN(A81,B81)</f>
-        <v>0</v>
-      </c>
-      <c r="F81" s="7"/>
+      <c r="E81" s="13">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A82" s="7">
+      <c r="A82">
         <v>1234.567</v>
       </c>
-      <c r="B82" s="7">
+      <c r="B82">
         <v>-0.5</v>
       </c>
-      <c r="C82" s="12">
-        <f>ROUND(A82,B82)</f>
+      <c r="C82" s="11">
+        <f t="shared" si="24"/>
         <v>1235</v>
       </c>
-      <c r="D82" s="12">
-        <f>ROUNDUP(A82,B82)</f>
+      <c r="D82" s="11">
+        <f t="shared" si="25"/>
         <v>1235</v>
       </c>
-      <c r="E82" s="14">
-        <f>ROUNDDOWN(A82,B82)</f>
+      <c r="E82" s="13">
+        <f t="shared" si="26"/>
         <v>1234</v>
       </c>
-      <c r="F82" s="7" t="s">
+      <c r="F82" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A83" s="7">
+      <c r="A83">
         <v>1234.567</v>
       </c>
-      <c r="B83" s="7">
+      <c r="B83">
         <v>-0.9</v>
       </c>
-      <c r="C83" s="12">
-        <f>ROUND(A83,B83)</f>
+      <c r="C83" s="11">
+        <f t="shared" si="24"/>
         <v>1235</v>
       </c>
-      <c r="D83" s="12">
-        <f>ROUNDUP(A83,B83)</f>
+      <c r="D83" s="11">
+        <f t="shared" si="25"/>
         <v>1235</v>
       </c>
-      <c r="E83" s="14">
-        <f>ROUNDDOWN(A83,B83)</f>
+      <c r="E83" s="13">
+        <f t="shared" si="26"/>
         <v>1234</v>
       </c>
-      <c r="F83" s="7"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A84" s="7">
+      <c r="A84">
         <v>1.7450000000000001</v>
       </c>
-      <c r="B84" s="7">
+      <c r="B84">
         <v>0.9</v>
       </c>
-      <c r="C84" s="12">
-        <f>ROUND(A84,B84)</f>
-        <v>2</v>
-      </c>
-      <c r="D84" s="12">
-        <f>ROUNDUP(A84,B84)</f>
-        <v>2</v>
-      </c>
-      <c r="E84" s="14">
-        <f>ROUNDDOWN(A84,B84)</f>
-        <v>1</v>
-      </c>
-      <c r="F84" s="7"/>
+      <c r="C84" s="11">
+        <f t="shared" si="24"/>
+        <v>2</v>
+      </c>
+      <c r="D84" s="11">
+        <f t="shared" si="25"/>
+        <v>2</v>
+      </c>
+      <c r="E84" s="13">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A85" s="7">
+      <c r="A85">
         <v>1.7450000000000001</v>
       </c>
-      <c r="B85" s="7" t="str">
+      <c r="B85" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="C85" s="12" t="e">
-        <f>ROUND(A85,B85)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D85" s="12" t="e">
-        <f>ROUNDUP(A85,B85)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E85" s="14" t="e">
-        <f>ROUNDDOWN(A85,B85)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F85" s="7" t="s">
+      <c r="C85" s="11" t="e">
+        <f t="shared" si="24"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D85" s="11" t="e">
+        <f t="shared" si="25"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E85" s="13" t="e">
+        <f t="shared" si="26"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F85" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A86" s="7" t="str">
+      <c r="A86" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="B86" s="7">
-        <v>2</v>
-      </c>
-      <c r="C86" s="12" t="e">
-        <f>ROUND(A86,B86)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D86" s="12" t="e">
-        <f>ROUNDUP(A86,B86)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E86" s="14" t="e">
-        <f>ROUNDDOWN(A86,B86)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F86" s="7" t="s">
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" s="11" t="e">
+        <f t="shared" si="24"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D86" s="11" t="e">
+        <f t="shared" si="25"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E86" s="13" t="e">
+        <f t="shared" si="26"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F86" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2466,19 +2451,19 @@
       <c r="B87">
         <v>2</v>
       </c>
-      <c r="C87" s="12">
-        <f>ROUND(A87,B87)</f>
+      <c r="C87" s="11">
+        <f t="shared" si="24"/>
         <v>1.75</v>
       </c>
-      <c r="D87" s="12">
-        <f>ROUNDUP(A87,B87)</f>
+      <c r="D87" s="11">
+        <f t="shared" si="25"/>
         <v>1.75</v>
       </c>
-      <c r="E87" s="14">
-        <f>ROUNDDOWN(A87,B87)</f>
+      <c r="E87" s="13">
+        <f t="shared" si="26"/>
         <v>1.74</v>
       </c>
-      <c r="F87" s="7" t="s">
+      <c r="F87" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2489,19 +2474,19 @@
       <c r="B88">
         <v>2</v>
       </c>
-      <c r="C88" s="12">
-        <f>ROUND(A88,B88)</f>
+      <c r="C88" s="11">
+        <f t="shared" si="24"/>
         <v>1.75</v>
       </c>
-      <c r="D88" s="12">
-        <f>ROUNDUP(A88,B88)</f>
+      <c r="D88" s="11">
+        <f t="shared" si="25"/>
         <v>1.75</v>
       </c>
-      <c r="E88" s="14">
-        <f>ROUNDDOWN(A88,B88)</f>
+      <c r="E88" s="13">
+        <f t="shared" si="26"/>
         <v>1.74</v>
       </c>
-      <c r="F88" s="7" t="s">
+      <c r="F88" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2512,19 +2497,19 @@
       <c r="B89">
         <v>1</v>
       </c>
-      <c r="C89" s="12">
-        <f>ROUND(A89,B89)</f>
+      <c r="C89" s="11">
+        <f t="shared" si="24"/>
         <v>0.5</v>
       </c>
-      <c r="D89" s="12">
-        <f>ROUNDUP(A89,B89)</f>
+      <c r="D89" s="11">
+        <f t="shared" si="25"/>
         <v>0.5</v>
       </c>
-      <c r="E89" s="14">
-        <f>ROUNDDOWN(A89,B89)</f>
+      <c r="E89" s="13">
+        <f t="shared" si="26"/>
         <v>0.5</v>
       </c>
-      <c r="F89" s="7" t="s">
+      <c r="F89" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2535,19 +2520,19 @@
       <c r="B90">
         <v>2</v>
       </c>
-      <c r="C90" s="12">
-        <f>ROUND(A90,B90)</f>
+      <c r="C90" s="11">
+        <f t="shared" si="24"/>
         <v>0.52</v>
       </c>
-      <c r="D90" s="12">
-        <f>ROUNDUP(A90,B90)</f>
+      <c r="D90" s="11">
+        <f t="shared" si="25"/>
         <v>0.53</v>
       </c>
-      <c r="E90" s="14">
-        <f>ROUNDDOWN(A90,B90)</f>
+      <c r="E90" s="13">
+        <f t="shared" si="26"/>
         <v>0.52</v>
       </c>
-      <c r="F90" s="7" t="s">
+      <c r="F90" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2558,235 +2543,225 @@
       <c r="B91">
         <v>0</v>
       </c>
-      <c r="C91" s="12" t="e">
-        <f>ROUND(A91,B91)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D91" s="12" t="e">
-        <f>ROUNDUP(A91,B91)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E91" s="14" t="e">
-        <f>ROUNDDOWN(A91,B91)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F91" s="7" t="s">
+      <c r="C91" s="11" t="e">
+        <f t="shared" si="24"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D91" s="11" t="e">
+        <f t="shared" si="25"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E91" s="13" t="e">
+        <f t="shared" si="26"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F91" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A92" s="7"/>
-      <c r="B92" s="7"/>
-      <c r="C92" s="12">
+      <c r="C92" s="11">
         <f>ROUND(TRUE,1)</f>
         <v>1</v>
       </c>
-      <c r="D92" s="12">
+      <c r="D92" s="11">
         <f>ROUNDUP(TRUE,1)</f>
         <v>1</v>
       </c>
-      <c r="E92" s="14">
+      <c r="E92" s="13">
         <f>ROUNDDOWN(TRUE,1)</f>
         <v>1</v>
       </c>
-      <c r="F92" s="7" t="s">
+      <c r="F92" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A93" s="7"/>
-      <c r="B93" s="7"/>
-      <c r="C93" s="12">
+      <c r="C93" s="11">
         <f>ROUND("1.745",2)</f>
         <v>1.75</v>
       </c>
-      <c r="D93" s="12">
+      <c r="D93" s="11">
         <f>ROUNDUP("1.745",2)</f>
         <v>1.75</v>
       </c>
-      <c r="E93" s="14">
+      <c r="E93" s="13">
         <f>ROUNDDOWN("1.745",2)</f>
         <v>1.74</v>
       </c>
-      <c r="F93" s="7" t="s">
+      <c r="F93" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A94" s="9">
+      <c r="A94" s="8">
         <f>TIME(12,30,0)</f>
         <v>0.52083333333333337</v>
       </c>
-      <c r="B94" s="7">
-        <v>2</v>
-      </c>
-      <c r="C94" s="12">
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" s="11">
         <f>ROUND(A94,B94)</f>
         <v>0.52</v>
       </c>
-      <c r="D94" s="12">
+      <c r="D94" s="11">
         <f>ROUNDUP(A94,B94)</f>
         <v>0.53</v>
       </c>
-      <c r="E94" s="14">
+      <c r="E94" s="13">
         <f>ROUNDDOWN(A94,B94)</f>
         <v>0.52</v>
       </c>
-      <c r="F94" s="7" t="s">
+      <c r="F94" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A95" s="8">
+      <c r="A95" s="7">
         <f>DATE(2026,1,1)+0.6</f>
         <v>46023.6</v>
       </c>
-      <c r="B95" s="7">
-        <v>0</v>
-      </c>
-      <c r="C95" s="12">
+      <c r="B95">
+        <v>0</v>
+      </c>
+      <c r="C95" s="11">
         <f>ROUND(A95,B95)</f>
         <v>46024</v>
       </c>
-      <c r="D95" s="12">
+      <c r="D95" s="11">
         <f>ROUNDUP(A95,B95)</f>
         <v>46024</v>
       </c>
-      <c r="E95" s="14">
+      <c r="E95" s="13">
         <f>ROUNDDOWN(A95,B95)</f>
         <v>46023</v>
       </c>
-      <c r="F95" s="7" t="s">
+      <c r="F95" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A96" s="7" t="e">
+      <c r="A96" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="B96" s="7">
-        <v>2</v>
-      </c>
-      <c r="C96" s="12" t="e">
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" s="11" t="e">
         <f>ROUND(A96,B96)</f>
         <v>#N/A</v>
       </c>
-      <c r="D96" s="12" t="e">
+      <c r="D96" s="11" t="e">
         <f>ROUNDUP(A96,B96)</f>
         <v>#N/A</v>
       </c>
-      <c r="E96" s="14" t="e">
+      <c r="E96" s="13" t="e">
         <f>ROUNDDOWN(A96,B96)</f>
         <v>#N/A</v>
       </c>
-      <c r="F96" s="7" t="s">
+      <c r="F96" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A97" s="7">
-        <v>2</v>
-      </c>
-      <c r="B97" s="7" t="e">
+      <c r="A97">
+        <v>2</v>
+      </c>
+      <c r="B97" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C97" s="12" t="e">
+      <c r="C97" s="11" t="e">
         <f>ROUND(A97,B97)</f>
         <v>#N/A</v>
       </c>
-      <c r="D97" s="12" t="e">
+      <c r="D97" s="11" t="e">
         <f>ROUNDUP(A97,B97)</f>
         <v>#N/A</v>
       </c>
-      <c r="E97" s="14" t="e">
+      <c r="E97" s="13" t="e">
         <f>ROUNDDOWN(A97,B97)</f>
         <v>#N/A</v>
       </c>
-      <c r="F97" s="7" t="s">
+      <c r="F97" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A98" s="7" t="e">
+      <c r="A98" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="B98" s="7" t="e">
+      <c r="B98" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C98" s="12" t="e">
+      <c r="C98" s="11" t="e">
         <f>ROUND(A98,B98)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D98" s="12" t="e">
+      <c r="D98" s="11" t="e">
         <f>ROUNDUP(A98,B98)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E98" s="14" t="e">
+      <c r="E98" s="13" t="e">
         <f>ROUNDDOWN(A98,B98)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F98" s="7" t="s">
+      <c r="F98" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A99" s="7"/>
-      <c r="B99" s="7"/>
-      <c r="C99" s="12" t="e">
+      <c r="C99" s="11" t="e">
         <f>ROUND(1.745,R7:R10)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D99" s="12" t="e">
+      <c r="D99" s="11" t="e">
         <f>ROUNDUP(1.745,R7:R10)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E99" s="14" t="e">
+      <c r="E99" s="13" t="e">
         <f>ROUNDDOWN(1.745,R7:R10)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F99" s="7" t="s">
+      <c r="F99" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A100" s="7"/>
-      <c r="B100" s="7"/>
-      <c r="C100" s="12" t="e">
+      <c r="C100" s="11" t="e">
         <f>ROUND(J3:M3,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D100" s="12" t="e">
+      <c r="D100" s="11" t="e">
         <f>ROUNDUP(J3:M3,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E100" s="14" t="e">
+      <c r="E100" s="13" t="e">
         <f>ROUNDDOWN(J3:M3,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F100" s="7" t="s">
+      <c r="F100" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A101" s="7"/>
-      <c r="B101" s="7"/>
-      <c r="C101" s="10" t="e">
+      <c r="C101" s="9" t="e">
         <f>ROUND(J2:K7,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D101" s="10" t="e">
+      <c r="D101" s="9" t="e">
         <f>ROUNDUP(J2:K7,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E101" s="11" t="e">
+      <c r="E101" s="10" t="e">
         <f>ROUNDDOWN(J2:K7,2)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F101" s="7" t="s">
+      <c r="F101" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>